<commit_message>
Implementar tematização dos pontos por data da última vistoria (Verde <= 7d, Amarelo 8-15d, Vermelho >= 16d)
</commit_message>
<xml_diff>
--- a/Visitas_Monitoramento_Sede.xlsx
+++ b/Visitas_Monitoramento_Sede.xlsx
@@ -520,7 +520,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P78"/>
+  <dimension ref="A1:R78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -571,35 +571,45 @@
       </c>
       <c r="J1" t="inlineStr">
         <is>
+          <t>STATUS_TEMATICO</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>DIAS_DESDE_ULTIMA_VISTORIA</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
           <t>TOTAL_VISTORIAS</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>ULTIMA_DATA</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>ULTIMA_PRESSAO</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>ULTIMAS_BANDEIRAS</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>ULTIMO_LARVA_PUPA</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>ULTIMO_INSETICIDA</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>ULTIMO_AVALIADOR</t>
         </is>
@@ -647,15 +657,21 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="J2" t="n">
-        <v>0</v>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Vermelho (Sem Vistoria)</t>
+        </is>
       </c>
       <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
+      <c r="L2" t="n">
+        <v>0</v>
+      </c>
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr"/>
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr"/>
+      <c r="R2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -699,15 +715,21 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="J3" t="n">
-        <v>0</v>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Vermelho (Sem Vistoria)</t>
+        </is>
       </c>
       <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
+      <c r="L3" t="n">
+        <v>0</v>
+      </c>
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr"/>
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr"/>
+      <c r="R3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -751,15 +773,21 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="J4" t="n">
-        <v>0</v>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Vermelho (Sem Vistoria)</t>
+        </is>
       </c>
       <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
+      <c r="L4" t="n">
+        <v>0</v>
+      </c>
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr"/>
       <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr"/>
+      <c r="R4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -803,15 +831,21 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="J5" t="n">
-        <v>0</v>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Vermelho (Sem Vistoria)</t>
+        </is>
       </c>
       <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
+      <c r="L5" t="n">
+        <v>0</v>
+      </c>
       <c r="M5" t="inlineStr"/>
       <c r="N5" t="inlineStr"/>
       <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr"/>
+      <c r="Q5" t="inlineStr"/>
+      <c r="R5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -855,15 +889,21 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="J6" t="n">
-        <v>0</v>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Vermelho (Sem Vistoria)</t>
+        </is>
       </c>
       <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
+      <c r="L6" t="n">
+        <v>0</v>
+      </c>
       <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr"/>
       <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr"/>
+      <c r="Q6" t="inlineStr"/>
+      <c r="R6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -907,15 +947,21 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="J7" t="n">
-        <v>0</v>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Vermelho (Sem Vistoria)</t>
+        </is>
       </c>
       <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
+      <c r="L7" t="n">
+        <v>0</v>
+      </c>
       <c r="M7" t="inlineStr"/>
       <c r="N7" t="inlineStr"/>
       <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr"/>
+      <c r="Q7" t="inlineStr"/>
+      <c r="R7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -959,15 +1005,21 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="J8" t="n">
-        <v>0</v>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Vermelho (Sem Vistoria)</t>
+        </is>
       </c>
       <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
+      <c r="L8" t="n">
+        <v>0</v>
+      </c>
       <c r="M8" t="inlineStr"/>
       <c r="N8" t="inlineStr"/>
       <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr"/>
+      <c r="Q8" t="inlineStr"/>
+      <c r="R8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1011,15 +1063,21 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="J9" t="n">
-        <v>0</v>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Vermelho (Sem Vistoria)</t>
+        </is>
       </c>
       <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
+      <c r="L9" t="n">
+        <v>0</v>
+      </c>
       <c r="M9" t="inlineStr"/>
       <c r="N9" t="inlineStr"/>
       <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr"/>
+      <c r="Q9" t="inlineStr"/>
+      <c r="R9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1063,15 +1121,21 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="J10" t="n">
-        <v>0</v>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Vermelho (Sem Vistoria)</t>
+        </is>
       </c>
       <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
+      <c r="L10" t="n">
+        <v>0</v>
+      </c>
       <c r="M10" t="inlineStr"/>
       <c r="N10" t="inlineStr"/>
       <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr"/>
+      <c r="Q10" t="inlineStr"/>
+      <c r="R10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1115,15 +1179,21 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="J11" t="n">
-        <v>0</v>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Vermelho (Sem Vistoria)</t>
+        </is>
       </c>
       <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
+      <c r="L11" t="n">
+        <v>0</v>
+      </c>
       <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr"/>
       <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr"/>
+      <c r="Q11" t="inlineStr"/>
+      <c r="R11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1167,15 +1237,21 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="J12" t="n">
-        <v>0</v>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Vermelho (Sem Vistoria)</t>
+        </is>
       </c>
       <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
+      <c r="L12" t="n">
+        <v>0</v>
+      </c>
       <c r="M12" t="inlineStr"/>
       <c r="N12" t="inlineStr"/>
       <c r="O12" t="inlineStr"/>
       <c r="P12" t="inlineStr"/>
+      <c r="Q12" t="inlineStr"/>
+      <c r="R12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1219,15 +1295,21 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="J13" t="n">
-        <v>0</v>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Vermelho (Sem Vistoria)</t>
+        </is>
       </c>
       <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
+      <c r="L13" t="n">
+        <v>0</v>
+      </c>
       <c r="M13" t="inlineStr"/>
       <c r="N13" t="inlineStr"/>
       <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr"/>
+      <c r="Q13" t="inlineStr"/>
+      <c r="R13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1271,15 +1353,21 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="J14" t="n">
-        <v>0</v>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Vermelho (Sem Vistoria)</t>
+        </is>
       </c>
       <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr"/>
+      <c r="L14" t="n">
+        <v>0</v>
+      </c>
       <c r="M14" t="inlineStr"/>
       <c r="N14" t="inlineStr"/>
       <c r="O14" t="inlineStr"/>
       <c r="P14" t="inlineStr"/>
+      <c r="Q14" t="inlineStr"/>
+      <c r="R14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1323,15 +1411,21 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="J15" t="n">
-        <v>0</v>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Vermelho (Sem Vistoria)</t>
+        </is>
       </c>
       <c r="K15" t="inlineStr"/>
-      <c r="L15" t="inlineStr"/>
+      <c r="L15" t="n">
+        <v>0</v>
+      </c>
       <c r="M15" t="inlineStr"/>
       <c r="N15" t="inlineStr"/>
       <c r="O15" t="inlineStr"/>
       <c r="P15" t="inlineStr"/>
+      <c r="Q15" t="inlineStr"/>
+      <c r="R15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1375,15 +1469,21 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="J16" t="n">
-        <v>0</v>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Vermelho (Sem Vistoria)</t>
+        </is>
       </c>
       <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr"/>
+      <c r="L16" t="n">
+        <v>0</v>
+      </c>
       <c r="M16" t="inlineStr"/>
       <c r="N16" t="inlineStr"/>
       <c r="O16" t="inlineStr"/>
       <c r="P16" t="inlineStr"/>
+      <c r="Q16" t="inlineStr"/>
+      <c r="R16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1427,15 +1527,21 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="J17" t="n">
-        <v>0</v>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Vermelho (Sem Vistoria)</t>
+        </is>
       </c>
       <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr"/>
+      <c r="L17" t="n">
+        <v>0</v>
+      </c>
       <c r="M17" t="inlineStr"/>
       <c r="N17" t="inlineStr"/>
       <c r="O17" t="inlineStr"/>
       <c r="P17" t="inlineStr"/>
+      <c r="Q17" t="inlineStr"/>
+      <c r="R17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1479,15 +1585,21 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="J18" t="n">
-        <v>0</v>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Vermelho (Sem Vistoria)</t>
+        </is>
       </c>
       <c r="K18" t="inlineStr"/>
-      <c r="L18" t="inlineStr"/>
+      <c r="L18" t="n">
+        <v>0</v>
+      </c>
       <c r="M18" t="inlineStr"/>
       <c r="N18" t="inlineStr"/>
       <c r="O18" t="inlineStr"/>
       <c r="P18" t="inlineStr"/>
+      <c r="Q18" t="inlineStr"/>
+      <c r="R18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1531,15 +1643,21 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="J19" t="n">
-        <v>0</v>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Vermelho (Sem Vistoria)</t>
+        </is>
       </c>
       <c r="K19" t="inlineStr"/>
-      <c r="L19" t="inlineStr"/>
+      <c r="L19" t="n">
+        <v>0</v>
+      </c>
       <c r="M19" t="inlineStr"/>
       <c r="N19" t="inlineStr"/>
       <c r="O19" t="inlineStr"/>
       <c r="P19" t="inlineStr"/>
+      <c r="Q19" t="inlineStr"/>
+      <c r="R19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1583,15 +1701,21 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="J20" t="n">
-        <v>0</v>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Vermelho (Sem Vistoria)</t>
+        </is>
       </c>
       <c r="K20" t="inlineStr"/>
-      <c r="L20" t="inlineStr"/>
+      <c r="L20" t="n">
+        <v>0</v>
+      </c>
       <c r="M20" t="inlineStr"/>
       <c r="N20" t="inlineStr"/>
       <c r="O20" t="inlineStr"/>
       <c r="P20" t="inlineStr"/>
+      <c r="Q20" t="inlineStr"/>
+      <c r="R20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1635,15 +1759,21 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="J21" t="n">
-        <v>0</v>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>Vermelho (Sem Vistoria)</t>
+        </is>
       </c>
       <c r="K21" t="inlineStr"/>
-      <c r="L21" t="inlineStr"/>
+      <c r="L21" t="n">
+        <v>0</v>
+      </c>
       <c r="M21" t="inlineStr"/>
       <c r="N21" t="inlineStr"/>
       <c r="O21" t="inlineStr"/>
       <c r="P21" t="inlineStr"/>
+      <c r="Q21" t="inlineStr"/>
+      <c r="R21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1687,15 +1817,21 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="J22" t="n">
-        <v>0</v>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Vermelho (Sem Vistoria)</t>
+        </is>
       </c>
       <c r="K22" t="inlineStr"/>
-      <c r="L22" t="inlineStr"/>
+      <c r="L22" t="n">
+        <v>0</v>
+      </c>
       <c r="M22" t="inlineStr"/>
       <c r="N22" t="inlineStr"/>
       <c r="O22" t="inlineStr"/>
       <c r="P22" t="inlineStr"/>
+      <c r="Q22" t="inlineStr"/>
+      <c r="R22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1739,15 +1875,21 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="J23" t="n">
-        <v>0</v>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Vermelho (Sem Vistoria)</t>
+        </is>
       </c>
       <c r="K23" t="inlineStr"/>
-      <c r="L23" t="inlineStr"/>
+      <c r="L23" t="n">
+        <v>0</v>
+      </c>
       <c r="M23" t="inlineStr"/>
       <c r="N23" t="inlineStr"/>
       <c r="O23" t="inlineStr"/>
       <c r="P23" t="inlineStr"/>
+      <c r="Q23" t="inlineStr"/>
+      <c r="R23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1791,15 +1933,21 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="J24" t="n">
-        <v>0</v>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Vermelho (Sem Vistoria)</t>
+        </is>
       </c>
       <c r="K24" t="inlineStr"/>
-      <c r="L24" t="inlineStr"/>
+      <c r="L24" t="n">
+        <v>0</v>
+      </c>
       <c r="M24" t="inlineStr"/>
       <c r="N24" t="inlineStr"/>
       <c r="O24" t="inlineStr"/>
       <c r="P24" t="inlineStr"/>
+      <c r="Q24" t="inlineStr"/>
+      <c r="R24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1843,15 +1991,21 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="J25" t="n">
-        <v>0</v>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>Vermelho (Sem Vistoria)</t>
+        </is>
       </c>
       <c r="K25" t="inlineStr"/>
-      <c r="L25" t="inlineStr"/>
+      <c r="L25" t="n">
+        <v>0</v>
+      </c>
       <c r="M25" t="inlineStr"/>
       <c r="N25" t="inlineStr"/>
       <c r="O25" t="inlineStr"/>
       <c r="P25" t="inlineStr"/>
+      <c r="Q25" t="inlineStr"/>
+      <c r="R25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1895,15 +2049,21 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="J26" t="n">
-        <v>0</v>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>Vermelho (Sem Vistoria)</t>
+        </is>
       </c>
       <c r="K26" t="inlineStr"/>
-      <c r="L26" t="inlineStr"/>
+      <c r="L26" t="n">
+        <v>0</v>
+      </c>
       <c r="M26" t="inlineStr"/>
       <c r="N26" t="inlineStr"/>
       <c r="O26" t="inlineStr"/>
       <c r="P26" t="inlineStr"/>
+      <c r="Q26" t="inlineStr"/>
+      <c r="R26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1947,15 +2107,21 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="J27" t="n">
-        <v>0</v>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>Vermelho (Sem Vistoria)</t>
+        </is>
       </c>
       <c r="K27" t="inlineStr"/>
-      <c r="L27" t="inlineStr"/>
+      <c r="L27" t="n">
+        <v>0</v>
+      </c>
       <c r="M27" t="inlineStr"/>
       <c r="N27" t="inlineStr"/>
       <c r="O27" t="inlineStr"/>
       <c r="P27" t="inlineStr"/>
+      <c r="Q27" t="inlineStr"/>
+      <c r="R27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1999,15 +2165,21 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="J28" t="n">
-        <v>0</v>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>Vermelho (Sem Vistoria)</t>
+        </is>
       </c>
       <c r="K28" t="inlineStr"/>
-      <c r="L28" t="inlineStr"/>
+      <c r="L28" t="n">
+        <v>0</v>
+      </c>
       <c r="M28" t="inlineStr"/>
       <c r="N28" t="inlineStr"/>
       <c r="O28" t="inlineStr"/>
       <c r="P28" t="inlineStr"/>
+      <c r="Q28" t="inlineStr"/>
+      <c r="R28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2051,15 +2223,21 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="J29" t="n">
-        <v>0</v>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>Vermelho (Sem Vistoria)</t>
+        </is>
       </c>
       <c r="K29" t="inlineStr"/>
-      <c r="L29" t="inlineStr"/>
+      <c r="L29" t="n">
+        <v>0</v>
+      </c>
       <c r="M29" t="inlineStr"/>
       <c r="N29" t="inlineStr"/>
       <c r="O29" t="inlineStr"/>
       <c r="P29" t="inlineStr"/>
+      <c r="Q29" t="inlineStr"/>
+      <c r="R29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2103,15 +2281,21 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="J30" t="n">
-        <v>0</v>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>Vermelho (Sem Vistoria)</t>
+        </is>
       </c>
       <c r="K30" t="inlineStr"/>
-      <c r="L30" t="inlineStr"/>
+      <c r="L30" t="n">
+        <v>0</v>
+      </c>
       <c r="M30" t="inlineStr"/>
       <c r="N30" t="inlineStr"/>
       <c r="O30" t="inlineStr"/>
       <c r="P30" t="inlineStr"/>
+      <c r="Q30" t="inlineStr"/>
+      <c r="R30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2155,15 +2339,21 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="J31" t="n">
-        <v>0</v>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>Vermelho (Sem Vistoria)</t>
+        </is>
       </c>
       <c r="K31" t="inlineStr"/>
-      <c r="L31" t="inlineStr"/>
+      <c r="L31" t="n">
+        <v>0</v>
+      </c>
       <c r="M31" t="inlineStr"/>
       <c r="N31" t="inlineStr"/>
       <c r="O31" t="inlineStr"/>
       <c r="P31" t="inlineStr"/>
+      <c r="Q31" t="inlineStr"/>
+      <c r="R31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2207,15 +2397,21 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="J32" t="n">
-        <v>0</v>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>Vermelho (Sem Vistoria)</t>
+        </is>
       </c>
       <c r="K32" t="inlineStr"/>
-      <c r="L32" t="inlineStr"/>
+      <c r="L32" t="n">
+        <v>0</v>
+      </c>
       <c r="M32" t="inlineStr"/>
       <c r="N32" t="inlineStr"/>
       <c r="O32" t="inlineStr"/>
       <c r="P32" t="inlineStr"/>
+      <c r="Q32" t="inlineStr"/>
+      <c r="R32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2259,15 +2455,21 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="J33" t="n">
-        <v>0</v>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>Vermelho (Sem Vistoria)</t>
+        </is>
       </c>
       <c r="K33" t="inlineStr"/>
-      <c r="L33" t="inlineStr"/>
+      <c r="L33" t="n">
+        <v>0</v>
+      </c>
       <c r="M33" t="inlineStr"/>
       <c r="N33" t="inlineStr"/>
       <c r="O33" t="inlineStr"/>
       <c r="P33" t="inlineStr"/>
+      <c r="Q33" t="inlineStr"/>
+      <c r="R33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2311,15 +2513,21 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="J34" t="n">
-        <v>0</v>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>Vermelho (Sem Vistoria)</t>
+        </is>
       </c>
       <c r="K34" t="inlineStr"/>
-      <c r="L34" t="inlineStr"/>
+      <c r="L34" t="n">
+        <v>0</v>
+      </c>
       <c r="M34" t="inlineStr"/>
       <c r="N34" t="inlineStr"/>
       <c r="O34" t="inlineStr"/>
       <c r="P34" t="inlineStr"/>
+      <c r="Q34" t="inlineStr"/>
+      <c r="R34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2363,15 +2571,21 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="J35" t="n">
-        <v>0</v>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>Vermelho (Sem Vistoria)</t>
+        </is>
       </c>
       <c r="K35" t="inlineStr"/>
-      <c r="L35" t="inlineStr"/>
+      <c r="L35" t="n">
+        <v>0</v>
+      </c>
       <c r="M35" t="inlineStr"/>
       <c r="N35" t="inlineStr"/>
       <c r="O35" t="inlineStr"/>
       <c r="P35" t="inlineStr"/>
+      <c r="Q35" t="inlineStr"/>
+      <c r="R35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2415,15 +2629,21 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="J36" t="n">
-        <v>0</v>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>Vermelho (Sem Vistoria)</t>
+        </is>
       </c>
       <c r="K36" t="inlineStr"/>
-      <c r="L36" t="inlineStr"/>
+      <c r="L36" t="n">
+        <v>0</v>
+      </c>
       <c r="M36" t="inlineStr"/>
       <c r="N36" t="inlineStr"/>
       <c r="O36" t="inlineStr"/>
       <c r="P36" t="inlineStr"/>
+      <c r="Q36" t="inlineStr"/>
+      <c r="R36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2467,15 +2687,21 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="J37" t="n">
-        <v>0</v>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>Vermelho (Sem Vistoria)</t>
+        </is>
       </c>
       <c r="K37" t="inlineStr"/>
-      <c r="L37" t="inlineStr"/>
+      <c r="L37" t="n">
+        <v>0</v>
+      </c>
       <c r="M37" t="inlineStr"/>
       <c r="N37" t="inlineStr"/>
       <c r="O37" t="inlineStr"/>
       <c r="P37" t="inlineStr"/>
+      <c r="Q37" t="inlineStr"/>
+      <c r="R37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2519,15 +2745,21 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="J38" t="n">
-        <v>0</v>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>Vermelho (Sem Vistoria)</t>
+        </is>
       </c>
       <c r="K38" t="inlineStr"/>
-      <c r="L38" t="inlineStr"/>
+      <c r="L38" t="n">
+        <v>0</v>
+      </c>
       <c r="M38" t="inlineStr"/>
       <c r="N38" t="inlineStr"/>
       <c r="O38" t="inlineStr"/>
       <c r="P38" t="inlineStr"/>
+      <c r="Q38" t="inlineStr"/>
+      <c r="R38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2571,15 +2803,21 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="J39" t="n">
-        <v>0</v>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>Vermelho (Sem Vistoria)</t>
+        </is>
       </c>
       <c r="K39" t="inlineStr"/>
-      <c r="L39" t="inlineStr"/>
+      <c r="L39" t="n">
+        <v>0</v>
+      </c>
       <c r="M39" t="inlineStr"/>
       <c r="N39" t="inlineStr"/>
       <c r="O39" t="inlineStr"/>
       <c r="P39" t="inlineStr"/>
+      <c r="Q39" t="inlineStr"/>
+      <c r="R39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2623,15 +2861,21 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="J40" t="n">
-        <v>0</v>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>Vermelho (Sem Vistoria)</t>
+        </is>
       </c>
       <c r="K40" t="inlineStr"/>
-      <c r="L40" t="inlineStr"/>
+      <c r="L40" t="n">
+        <v>0</v>
+      </c>
       <c r="M40" t="inlineStr"/>
       <c r="N40" t="inlineStr"/>
       <c r="O40" t="inlineStr"/>
       <c r="P40" t="inlineStr"/>
+      <c r="Q40" t="inlineStr"/>
+      <c r="R40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2675,15 +2919,21 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="J41" t="n">
-        <v>0</v>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>Vermelho (Sem Vistoria)</t>
+        </is>
       </c>
       <c r="K41" t="inlineStr"/>
-      <c r="L41" t="inlineStr"/>
+      <c r="L41" t="n">
+        <v>0</v>
+      </c>
       <c r="M41" t="inlineStr"/>
       <c r="N41" t="inlineStr"/>
       <c r="O41" t="inlineStr"/>
       <c r="P41" t="inlineStr"/>
+      <c r="Q41" t="inlineStr"/>
+      <c r="R41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2727,15 +2977,21 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="J42" t="n">
-        <v>0</v>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>Vermelho (Sem Vistoria)</t>
+        </is>
       </c>
       <c r="K42" t="inlineStr"/>
-      <c r="L42" t="inlineStr"/>
+      <c r="L42" t="n">
+        <v>0</v>
+      </c>
       <c r="M42" t="inlineStr"/>
       <c r="N42" t="inlineStr"/>
       <c r="O42" t="inlineStr"/>
       <c r="P42" t="inlineStr"/>
+      <c r="Q42" t="inlineStr"/>
+      <c r="R42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2779,15 +3035,21 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="J43" t="n">
-        <v>0</v>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>Vermelho (Sem Vistoria)</t>
+        </is>
       </c>
       <c r="K43" t="inlineStr"/>
-      <c r="L43" t="inlineStr"/>
+      <c r="L43" t="n">
+        <v>0</v>
+      </c>
       <c r="M43" t="inlineStr"/>
       <c r="N43" t="inlineStr"/>
       <c r="O43" t="inlineStr"/>
       <c r="P43" t="inlineStr"/>
+      <c r="Q43" t="inlineStr"/>
+      <c r="R43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2831,15 +3093,21 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="J44" t="n">
-        <v>0</v>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>Vermelho (Sem Vistoria)</t>
+        </is>
       </c>
       <c r="K44" t="inlineStr"/>
-      <c r="L44" t="inlineStr"/>
+      <c r="L44" t="n">
+        <v>0</v>
+      </c>
       <c r="M44" t="inlineStr"/>
       <c r="N44" t="inlineStr"/>
       <c r="O44" t="inlineStr"/>
       <c r="P44" t="inlineStr"/>
+      <c r="Q44" t="inlineStr"/>
+      <c r="R44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2883,15 +3151,21 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="J45" t="n">
-        <v>0</v>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>Vermelho (Sem Vistoria)</t>
+        </is>
       </c>
       <c r="K45" t="inlineStr"/>
-      <c r="L45" t="inlineStr"/>
+      <c r="L45" t="n">
+        <v>0</v>
+      </c>
       <c r="M45" t="inlineStr"/>
       <c r="N45" t="inlineStr"/>
       <c r="O45" t="inlineStr"/>
       <c r="P45" t="inlineStr"/>
+      <c r="Q45" t="inlineStr"/>
+      <c r="R45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2935,15 +3209,21 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="J46" t="n">
-        <v>0</v>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>Vermelho (Sem Vistoria)</t>
+        </is>
       </c>
       <c r="K46" t="inlineStr"/>
-      <c r="L46" t="inlineStr"/>
+      <c r="L46" t="n">
+        <v>0</v>
+      </c>
       <c r="M46" t="inlineStr"/>
       <c r="N46" t="inlineStr"/>
       <c r="O46" t="inlineStr"/>
       <c r="P46" t="inlineStr"/>
+      <c r="Q46" t="inlineStr"/>
+      <c r="R46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2987,15 +3267,21 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="J47" t="n">
-        <v>0</v>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>Vermelho (Sem Vistoria)</t>
+        </is>
       </c>
       <c r="K47" t="inlineStr"/>
-      <c r="L47" t="inlineStr"/>
+      <c r="L47" t="n">
+        <v>0</v>
+      </c>
       <c r="M47" t="inlineStr"/>
       <c r="N47" t="inlineStr"/>
       <c r="O47" t="inlineStr"/>
       <c r="P47" t="inlineStr"/>
+      <c r="Q47" t="inlineStr"/>
+      <c r="R47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -3039,15 +3325,21 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="J48" t="n">
-        <v>0</v>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>Vermelho (Sem Vistoria)</t>
+        </is>
       </c>
       <c r="K48" t="inlineStr"/>
-      <c r="L48" t="inlineStr"/>
+      <c r="L48" t="n">
+        <v>0</v>
+      </c>
       <c r="M48" t="inlineStr"/>
       <c r="N48" t="inlineStr"/>
       <c r="O48" t="inlineStr"/>
       <c r="P48" t="inlineStr"/>
+      <c r="Q48" t="inlineStr"/>
+      <c r="R48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -3091,15 +3383,21 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="J49" t="n">
-        <v>0</v>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>Vermelho (Sem Vistoria)</t>
+        </is>
       </c>
       <c r="K49" t="inlineStr"/>
-      <c r="L49" t="inlineStr"/>
+      <c r="L49" t="n">
+        <v>0</v>
+      </c>
       <c r="M49" t="inlineStr"/>
       <c r="N49" t="inlineStr"/>
       <c r="O49" t="inlineStr"/>
       <c r="P49" t="inlineStr"/>
+      <c r="Q49" t="inlineStr"/>
+      <c r="R49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -3143,15 +3441,21 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="J50" t="n">
-        <v>0</v>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>Vermelho (Sem Vistoria)</t>
+        </is>
       </c>
       <c r="K50" t="inlineStr"/>
-      <c r="L50" t="inlineStr"/>
+      <c r="L50" t="n">
+        <v>0</v>
+      </c>
       <c r="M50" t="inlineStr"/>
       <c r="N50" t="inlineStr"/>
       <c r="O50" t="inlineStr"/>
       <c r="P50" t="inlineStr"/>
+      <c r="Q50" t="inlineStr"/>
+      <c r="R50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -3195,15 +3499,21 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="J51" t="n">
-        <v>0</v>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>Vermelho (Sem Vistoria)</t>
+        </is>
       </c>
       <c r="K51" t="inlineStr"/>
-      <c r="L51" t="inlineStr"/>
+      <c r="L51" t="n">
+        <v>0</v>
+      </c>
       <c r="M51" t="inlineStr"/>
       <c r="N51" t="inlineStr"/>
       <c r="O51" t="inlineStr"/>
       <c r="P51" t="inlineStr"/>
+      <c r="Q51" t="inlineStr"/>
+      <c r="R51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -3247,15 +3557,21 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="J52" t="n">
-        <v>0</v>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>Vermelho (Sem Vistoria)</t>
+        </is>
       </c>
       <c r="K52" t="inlineStr"/>
-      <c r="L52" t="inlineStr"/>
+      <c r="L52" t="n">
+        <v>0</v>
+      </c>
       <c r="M52" t="inlineStr"/>
       <c r="N52" t="inlineStr"/>
       <c r="O52" t="inlineStr"/>
       <c r="P52" t="inlineStr"/>
+      <c r="Q52" t="inlineStr"/>
+      <c r="R52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -3299,15 +3615,21 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="J53" t="n">
-        <v>0</v>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>Vermelho (Sem Vistoria)</t>
+        </is>
       </c>
       <c r="K53" t="inlineStr"/>
-      <c r="L53" t="inlineStr"/>
+      <c r="L53" t="n">
+        <v>0</v>
+      </c>
       <c r="M53" t="inlineStr"/>
       <c r="N53" t="inlineStr"/>
       <c r="O53" t="inlineStr"/>
       <c r="P53" t="inlineStr"/>
+      <c r="Q53" t="inlineStr"/>
+      <c r="R53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -3351,15 +3673,21 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="J54" t="n">
-        <v>0</v>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>Vermelho (Sem Vistoria)</t>
+        </is>
       </c>
       <c r="K54" t="inlineStr"/>
-      <c r="L54" t="inlineStr"/>
+      <c r="L54" t="n">
+        <v>0</v>
+      </c>
       <c r="M54" t="inlineStr"/>
       <c r="N54" t="inlineStr"/>
       <c r="O54" t="inlineStr"/>
       <c r="P54" t="inlineStr"/>
+      <c r="Q54" t="inlineStr"/>
+      <c r="R54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -3403,15 +3731,21 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="J55" t="n">
-        <v>0</v>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>Vermelho (Sem Vistoria)</t>
+        </is>
       </c>
       <c r="K55" t="inlineStr"/>
-      <c r="L55" t="inlineStr"/>
+      <c r="L55" t="n">
+        <v>0</v>
+      </c>
       <c r="M55" t="inlineStr"/>
       <c r="N55" t="inlineStr"/>
       <c r="O55" t="inlineStr"/>
       <c r="P55" t="inlineStr"/>
+      <c r="Q55" t="inlineStr"/>
+      <c r="R55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -3455,15 +3789,21 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="J56" t="n">
-        <v>0</v>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>Vermelho (Sem Vistoria)</t>
+        </is>
       </c>
       <c r="K56" t="inlineStr"/>
-      <c r="L56" t="inlineStr"/>
+      <c r="L56" t="n">
+        <v>0</v>
+      </c>
       <c r="M56" t="inlineStr"/>
       <c r="N56" t="inlineStr"/>
       <c r="O56" t="inlineStr"/>
       <c r="P56" t="inlineStr"/>
+      <c r="Q56" t="inlineStr"/>
+      <c r="R56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -3507,15 +3847,21 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="J57" t="n">
-        <v>0</v>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>Vermelho (Sem Vistoria)</t>
+        </is>
       </c>
       <c r="K57" t="inlineStr"/>
-      <c r="L57" t="inlineStr"/>
+      <c r="L57" t="n">
+        <v>0</v>
+      </c>
       <c r="M57" t="inlineStr"/>
       <c r="N57" t="inlineStr"/>
       <c r="O57" t="inlineStr"/>
       <c r="P57" t="inlineStr"/>
+      <c r="Q57" t="inlineStr"/>
+      <c r="R57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -3559,15 +3905,21 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="J58" t="n">
-        <v>0</v>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>Vermelho (Sem Vistoria)</t>
+        </is>
       </c>
       <c r="K58" t="inlineStr"/>
-      <c r="L58" t="inlineStr"/>
+      <c r="L58" t="n">
+        <v>0</v>
+      </c>
       <c r="M58" t="inlineStr"/>
       <c r="N58" t="inlineStr"/>
       <c r="O58" t="inlineStr"/>
       <c r="P58" t="inlineStr"/>
+      <c r="Q58" t="inlineStr"/>
+      <c r="R58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -3611,15 +3963,21 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="J59" t="n">
-        <v>0</v>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>Vermelho (Sem Vistoria)</t>
+        </is>
       </c>
       <c r="K59" t="inlineStr"/>
-      <c r="L59" t="inlineStr"/>
+      <c r="L59" t="n">
+        <v>0</v>
+      </c>
       <c r="M59" t="inlineStr"/>
       <c r="N59" t="inlineStr"/>
       <c r="O59" t="inlineStr"/>
       <c r="P59" t="inlineStr"/>
+      <c r="Q59" t="inlineStr"/>
+      <c r="R59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -3663,15 +4021,21 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="J60" t="n">
-        <v>0</v>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>Vermelho (Sem Vistoria)</t>
+        </is>
       </c>
       <c r="K60" t="inlineStr"/>
-      <c r="L60" t="inlineStr"/>
+      <c r="L60" t="n">
+        <v>0</v>
+      </c>
       <c r="M60" t="inlineStr"/>
       <c r="N60" t="inlineStr"/>
       <c r="O60" t="inlineStr"/>
       <c r="P60" t="inlineStr"/>
+      <c r="Q60" t="inlineStr"/>
+      <c r="R60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -3715,15 +4079,21 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="J61" t="n">
-        <v>0</v>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>Vermelho (Sem Vistoria)</t>
+        </is>
       </c>
       <c r="K61" t="inlineStr"/>
-      <c r="L61" t="inlineStr"/>
+      <c r="L61" t="n">
+        <v>0</v>
+      </c>
       <c r="M61" t="inlineStr"/>
       <c r="N61" t="inlineStr"/>
       <c r="O61" t="inlineStr"/>
       <c r="P61" t="inlineStr"/>
+      <c r="Q61" t="inlineStr"/>
+      <c r="R61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -3767,15 +4137,21 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="J62" t="n">
-        <v>0</v>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>Vermelho (Sem Vistoria)</t>
+        </is>
       </c>
       <c r="K62" t="inlineStr"/>
-      <c r="L62" t="inlineStr"/>
+      <c r="L62" t="n">
+        <v>0</v>
+      </c>
       <c r="M62" t="inlineStr"/>
       <c r="N62" t="inlineStr"/>
       <c r="O62" t="inlineStr"/>
       <c r="P62" t="inlineStr"/>
+      <c r="Q62" t="inlineStr"/>
+      <c r="R62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -3819,15 +4195,21 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="J63" t="n">
-        <v>0</v>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>Vermelho (Sem Vistoria)</t>
+        </is>
       </c>
       <c r="K63" t="inlineStr"/>
-      <c r="L63" t="inlineStr"/>
+      <c r="L63" t="n">
+        <v>0</v>
+      </c>
       <c r="M63" t="inlineStr"/>
       <c r="N63" t="inlineStr"/>
       <c r="O63" t="inlineStr"/>
       <c r="P63" t="inlineStr"/>
+      <c r="Q63" t="inlineStr"/>
+      <c r="R63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -3871,15 +4253,21 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="J64" t="n">
-        <v>0</v>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>Vermelho (Sem Vistoria)</t>
+        </is>
       </c>
       <c r="K64" t="inlineStr"/>
-      <c r="L64" t="inlineStr"/>
+      <c r="L64" t="n">
+        <v>0</v>
+      </c>
       <c r="M64" t="inlineStr"/>
       <c r="N64" t="inlineStr"/>
       <c r="O64" t="inlineStr"/>
       <c r="P64" t="inlineStr"/>
+      <c r="Q64" t="inlineStr"/>
+      <c r="R64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -3923,15 +4311,21 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="J65" t="n">
-        <v>0</v>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>Vermelho (Sem Vistoria)</t>
+        </is>
       </c>
       <c r="K65" t="inlineStr"/>
-      <c r="L65" t="inlineStr"/>
+      <c r="L65" t="n">
+        <v>0</v>
+      </c>
       <c r="M65" t="inlineStr"/>
       <c r="N65" t="inlineStr"/>
       <c r="O65" t="inlineStr"/>
       <c r="P65" t="inlineStr"/>
+      <c r="Q65" t="inlineStr"/>
+      <c r="R65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -3975,15 +4369,21 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="J66" t="n">
-        <v>0</v>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>Vermelho (Sem Vistoria)</t>
+        </is>
       </c>
       <c r="K66" t="inlineStr"/>
-      <c r="L66" t="inlineStr"/>
+      <c r="L66" t="n">
+        <v>0</v>
+      </c>
       <c r="M66" t="inlineStr"/>
       <c r="N66" t="inlineStr"/>
       <c r="O66" t="inlineStr"/>
       <c r="P66" t="inlineStr"/>
+      <c r="Q66" t="inlineStr"/>
+      <c r="R66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -4027,15 +4427,21 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="J67" t="n">
-        <v>0</v>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>Vermelho (Sem Vistoria)</t>
+        </is>
       </c>
       <c r="K67" t="inlineStr"/>
-      <c r="L67" t="inlineStr"/>
+      <c r="L67" t="n">
+        <v>0</v>
+      </c>
       <c r="M67" t="inlineStr"/>
       <c r="N67" t="inlineStr"/>
       <c r="O67" t="inlineStr"/>
       <c r="P67" t="inlineStr"/>
+      <c r="Q67" t="inlineStr"/>
+      <c r="R67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -4079,15 +4485,21 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="J68" t="n">
-        <v>0</v>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>Vermelho (Sem Vistoria)</t>
+        </is>
       </c>
       <c r="K68" t="inlineStr"/>
-      <c r="L68" t="inlineStr"/>
+      <c r="L68" t="n">
+        <v>0</v>
+      </c>
       <c r="M68" t="inlineStr"/>
       <c r="N68" t="inlineStr"/>
       <c r="O68" t="inlineStr"/>
       <c r="P68" t="inlineStr"/>
+      <c r="Q68" t="inlineStr"/>
+      <c r="R68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -4131,15 +4543,21 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="J69" t="n">
-        <v>0</v>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>Vermelho (Sem Vistoria)</t>
+        </is>
       </c>
       <c r="K69" t="inlineStr"/>
-      <c r="L69" t="inlineStr"/>
+      <c r="L69" t="n">
+        <v>0</v>
+      </c>
       <c r="M69" t="inlineStr"/>
       <c r="N69" t="inlineStr"/>
       <c r="O69" t="inlineStr"/>
       <c r="P69" t="inlineStr"/>
+      <c r="Q69" t="inlineStr"/>
+      <c r="R69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -4183,15 +4601,21 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="J70" t="n">
-        <v>0</v>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>Vermelho (Sem Vistoria)</t>
+        </is>
       </c>
       <c r="K70" t="inlineStr"/>
-      <c r="L70" t="inlineStr"/>
+      <c r="L70" t="n">
+        <v>0</v>
+      </c>
       <c r="M70" t="inlineStr"/>
       <c r="N70" t="inlineStr"/>
       <c r="O70" t="inlineStr"/>
       <c r="P70" t="inlineStr"/>
+      <c r="Q70" t="inlineStr"/>
+      <c r="R70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -4235,15 +4659,21 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="J71" t="n">
-        <v>0</v>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>Vermelho (Sem Vistoria)</t>
+        </is>
       </c>
       <c r="K71" t="inlineStr"/>
-      <c r="L71" t="inlineStr"/>
+      <c r="L71" t="n">
+        <v>0</v>
+      </c>
       <c r="M71" t="inlineStr"/>
       <c r="N71" t="inlineStr"/>
       <c r="O71" t="inlineStr"/>
       <c r="P71" t="inlineStr"/>
+      <c r="Q71" t="inlineStr"/>
+      <c r="R71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -4287,15 +4717,21 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="J72" t="n">
-        <v>0</v>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>Vermelho (Sem Vistoria)</t>
+        </is>
       </c>
       <c r="K72" t="inlineStr"/>
-      <c r="L72" t="inlineStr"/>
+      <c r="L72" t="n">
+        <v>0</v>
+      </c>
       <c r="M72" t="inlineStr"/>
       <c r="N72" t="inlineStr"/>
       <c r="O72" t="inlineStr"/>
       <c r="P72" t="inlineStr"/>
+      <c r="Q72" t="inlineStr"/>
+      <c r="R72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -4339,15 +4775,21 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="J73" t="n">
-        <v>0</v>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>Vermelho (Sem Vistoria)</t>
+        </is>
       </c>
       <c r="K73" t="inlineStr"/>
-      <c r="L73" t="inlineStr"/>
+      <c r="L73" t="n">
+        <v>0</v>
+      </c>
       <c r="M73" t="inlineStr"/>
       <c r="N73" t="inlineStr"/>
       <c r="O73" t="inlineStr"/>
       <c r="P73" t="inlineStr"/>
+      <c r="Q73" t="inlineStr"/>
+      <c r="R73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -4391,15 +4833,21 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="J74" t="n">
-        <v>0</v>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>Vermelho (Sem Vistoria)</t>
+        </is>
       </c>
       <c r="K74" t="inlineStr"/>
-      <c r="L74" t="inlineStr"/>
+      <c r="L74" t="n">
+        <v>0</v>
+      </c>
       <c r="M74" t="inlineStr"/>
       <c r="N74" t="inlineStr"/>
       <c r="O74" t="inlineStr"/>
       <c r="P74" t="inlineStr"/>
+      <c r="Q74" t="inlineStr"/>
+      <c r="R74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -4443,15 +4891,21 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="J75" t="n">
-        <v>0</v>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>Vermelho (Sem Vistoria)</t>
+        </is>
       </c>
       <c r="K75" t="inlineStr"/>
-      <c r="L75" t="inlineStr"/>
+      <c r="L75" t="n">
+        <v>0</v>
+      </c>
       <c r="M75" t="inlineStr"/>
       <c r="N75" t="inlineStr"/>
       <c r="O75" t="inlineStr"/>
       <c r="P75" t="inlineStr"/>
+      <c r="Q75" t="inlineStr"/>
+      <c r="R75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -4495,15 +4949,21 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="J76" t="n">
-        <v>0</v>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>Vermelho (Sem Vistoria)</t>
+        </is>
       </c>
       <c r="K76" t="inlineStr"/>
-      <c r="L76" t="inlineStr"/>
+      <c r="L76" t="n">
+        <v>0</v>
+      </c>
       <c r="M76" t="inlineStr"/>
       <c r="N76" t="inlineStr"/>
       <c r="O76" t="inlineStr"/>
       <c r="P76" t="inlineStr"/>
+      <c r="Q76" t="inlineStr"/>
+      <c r="R76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -4547,15 +5007,21 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="J77" t="n">
-        <v>0</v>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>Vermelho (Sem Vistoria)</t>
+        </is>
       </c>
       <c r="K77" t="inlineStr"/>
-      <c r="L77" t="inlineStr"/>
+      <c r="L77" t="n">
+        <v>0</v>
+      </c>
       <c r="M77" t="inlineStr"/>
       <c r="N77" t="inlineStr"/>
       <c r="O77" t="inlineStr"/>
       <c r="P77" t="inlineStr"/>
+      <c r="Q77" t="inlineStr"/>
+      <c r="R77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -4599,15 +5065,21 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="J78" t="n">
-        <v>0</v>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>Vermelho (Sem Vistoria)</t>
+        </is>
       </c>
       <c r="K78" t="inlineStr"/>
-      <c r="L78" t="inlineStr"/>
+      <c r="L78" t="n">
+        <v>0</v>
+      </c>
       <c r="M78" t="inlineStr"/>
       <c r="N78" t="inlineStr"/>
       <c r="O78" t="inlineStr"/>
       <c r="P78" t="inlineStr"/>
+      <c r="Q78" t="inlineStr"/>
+      <c r="R78" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Formulario: matricula flexivel ate 6 digitos, remover foto e adicionar possiveis causadores (Torta, Vinhaca, Outro)
</commit_message>
<xml_diff>
--- a/Visitas_Monitoramento_Sede.xlsx
+++ b/Visitas_Monitoramento_Sede.xlsx
@@ -485,12 +485,12 @@
       </c>
       <c r="N1" t="inlineStr">
         <is>
+          <t>POSSIVEIS_CAUSADORES</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
           <t>OBSERVACOES</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>FOTO</t>
         </is>
       </c>
       <c r="P1" t="inlineStr">
@@ -520,7 +520,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R78"/>
+  <dimension ref="A1:S78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -610,6 +610,11 @@
         </is>
       </c>
       <c r="R1" t="inlineStr">
+        <is>
+          <t>ULTIMOS_CAUSADORES</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
         <is>
           <t>ULTIMO_AVALIADOR</t>
         </is>
@@ -672,6 +677,7 @@
       <c r="P2" t="inlineStr"/>
       <c r="Q2" t="inlineStr"/>
       <c r="R2" t="inlineStr"/>
+      <c r="S2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -730,6 +736,7 @@
       <c r="P3" t="inlineStr"/>
       <c r="Q3" t="inlineStr"/>
       <c r="R3" t="inlineStr"/>
+      <c r="S3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -788,6 +795,7 @@
       <c r="P4" t="inlineStr"/>
       <c r="Q4" t="inlineStr"/>
       <c r="R4" t="inlineStr"/>
+      <c r="S4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -846,6 +854,7 @@
       <c r="P5" t="inlineStr"/>
       <c r="Q5" t="inlineStr"/>
       <c r="R5" t="inlineStr"/>
+      <c r="S5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -904,6 +913,7 @@
       <c r="P6" t="inlineStr"/>
       <c r="Q6" t="inlineStr"/>
       <c r="R6" t="inlineStr"/>
+      <c r="S6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -962,6 +972,7 @@
       <c r="P7" t="inlineStr"/>
       <c r="Q7" t="inlineStr"/>
       <c r="R7" t="inlineStr"/>
+      <c r="S7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1020,6 +1031,7 @@
       <c r="P8" t="inlineStr"/>
       <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr"/>
+      <c r="S8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1078,6 +1090,7 @@
       <c r="P9" t="inlineStr"/>
       <c r="Q9" t="inlineStr"/>
       <c r="R9" t="inlineStr"/>
+      <c r="S9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1136,6 +1149,7 @@
       <c r="P10" t="inlineStr"/>
       <c r="Q10" t="inlineStr"/>
       <c r="R10" t="inlineStr"/>
+      <c r="S10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1194,6 +1208,7 @@
       <c r="P11" t="inlineStr"/>
       <c r="Q11" t="inlineStr"/>
       <c r="R11" t="inlineStr"/>
+      <c r="S11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1252,6 +1267,7 @@
       <c r="P12" t="inlineStr"/>
       <c r="Q12" t="inlineStr"/>
       <c r="R12" t="inlineStr"/>
+      <c r="S12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1310,6 +1326,7 @@
       <c r="P13" t="inlineStr"/>
       <c r="Q13" t="inlineStr"/>
       <c r="R13" t="inlineStr"/>
+      <c r="S13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1368,6 +1385,7 @@
       <c r="P14" t="inlineStr"/>
       <c r="Q14" t="inlineStr"/>
       <c r="R14" t="inlineStr"/>
+      <c r="S14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1426,6 +1444,7 @@
       <c r="P15" t="inlineStr"/>
       <c r="Q15" t="inlineStr"/>
       <c r="R15" t="inlineStr"/>
+      <c r="S15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1484,6 +1503,7 @@
       <c r="P16" t="inlineStr"/>
       <c r="Q16" t="inlineStr"/>
       <c r="R16" t="inlineStr"/>
+      <c r="S16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1542,6 +1562,7 @@
       <c r="P17" t="inlineStr"/>
       <c r="Q17" t="inlineStr"/>
       <c r="R17" t="inlineStr"/>
+      <c r="S17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1600,6 +1621,7 @@
       <c r="P18" t="inlineStr"/>
       <c r="Q18" t="inlineStr"/>
       <c r="R18" t="inlineStr"/>
+      <c r="S18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1658,6 +1680,7 @@
       <c r="P19" t="inlineStr"/>
       <c r="Q19" t="inlineStr"/>
       <c r="R19" t="inlineStr"/>
+      <c r="S19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1716,6 +1739,7 @@
       <c r="P20" t="inlineStr"/>
       <c r="Q20" t="inlineStr"/>
       <c r="R20" t="inlineStr"/>
+      <c r="S20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1774,6 +1798,7 @@
       <c r="P21" t="inlineStr"/>
       <c r="Q21" t="inlineStr"/>
       <c r="R21" t="inlineStr"/>
+      <c r="S21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1832,6 +1857,7 @@
       <c r="P22" t="inlineStr"/>
       <c r="Q22" t="inlineStr"/>
       <c r="R22" t="inlineStr"/>
+      <c r="S22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1890,6 +1916,7 @@
       <c r="P23" t="inlineStr"/>
       <c r="Q23" t="inlineStr"/>
       <c r="R23" t="inlineStr"/>
+      <c r="S23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1948,6 +1975,7 @@
       <c r="P24" t="inlineStr"/>
       <c r="Q24" t="inlineStr"/>
       <c r="R24" t="inlineStr"/>
+      <c r="S24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2006,6 +2034,7 @@
       <c r="P25" t="inlineStr"/>
       <c r="Q25" t="inlineStr"/>
       <c r="R25" t="inlineStr"/>
+      <c r="S25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2064,6 +2093,7 @@
       <c r="P26" t="inlineStr"/>
       <c r="Q26" t="inlineStr"/>
       <c r="R26" t="inlineStr"/>
+      <c r="S26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2122,6 +2152,7 @@
       <c r="P27" t="inlineStr"/>
       <c r="Q27" t="inlineStr"/>
       <c r="R27" t="inlineStr"/>
+      <c r="S27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2180,6 +2211,7 @@
       <c r="P28" t="inlineStr"/>
       <c r="Q28" t="inlineStr"/>
       <c r="R28" t="inlineStr"/>
+      <c r="S28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2238,6 +2270,7 @@
       <c r="P29" t="inlineStr"/>
       <c r="Q29" t="inlineStr"/>
       <c r="R29" t="inlineStr"/>
+      <c r="S29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2296,6 +2329,7 @@
       <c r="P30" t="inlineStr"/>
       <c r="Q30" t="inlineStr"/>
       <c r="R30" t="inlineStr"/>
+      <c r="S30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2354,6 +2388,7 @@
       <c r="P31" t="inlineStr"/>
       <c r="Q31" t="inlineStr"/>
       <c r="R31" t="inlineStr"/>
+      <c r="S31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2412,6 +2447,7 @@
       <c r="P32" t="inlineStr"/>
       <c r="Q32" t="inlineStr"/>
       <c r="R32" t="inlineStr"/>
+      <c r="S32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2470,6 +2506,7 @@
       <c r="P33" t="inlineStr"/>
       <c r="Q33" t="inlineStr"/>
       <c r="R33" t="inlineStr"/>
+      <c r="S33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2528,6 +2565,7 @@
       <c r="P34" t="inlineStr"/>
       <c r="Q34" t="inlineStr"/>
       <c r="R34" t="inlineStr"/>
+      <c r="S34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2586,6 +2624,7 @@
       <c r="P35" t="inlineStr"/>
       <c r="Q35" t="inlineStr"/>
       <c r="R35" t="inlineStr"/>
+      <c r="S35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2644,6 +2683,7 @@
       <c r="P36" t="inlineStr"/>
       <c r="Q36" t="inlineStr"/>
       <c r="R36" t="inlineStr"/>
+      <c r="S36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2702,6 +2742,7 @@
       <c r="P37" t="inlineStr"/>
       <c r="Q37" t="inlineStr"/>
       <c r="R37" t="inlineStr"/>
+      <c r="S37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2760,6 +2801,7 @@
       <c r="P38" t="inlineStr"/>
       <c r="Q38" t="inlineStr"/>
       <c r="R38" t="inlineStr"/>
+      <c r="S38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2818,6 +2860,7 @@
       <c r="P39" t="inlineStr"/>
       <c r="Q39" t="inlineStr"/>
       <c r="R39" t="inlineStr"/>
+      <c r="S39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2876,6 +2919,7 @@
       <c r="P40" t="inlineStr"/>
       <c r="Q40" t="inlineStr"/>
       <c r="R40" t="inlineStr"/>
+      <c r="S40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2934,6 +2978,7 @@
       <c r="P41" t="inlineStr"/>
       <c r="Q41" t="inlineStr"/>
       <c r="R41" t="inlineStr"/>
+      <c r="S41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2992,6 +3037,7 @@
       <c r="P42" t="inlineStr"/>
       <c r="Q42" t="inlineStr"/>
       <c r="R42" t="inlineStr"/>
+      <c r="S42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -3050,6 +3096,7 @@
       <c r="P43" t="inlineStr"/>
       <c r="Q43" t="inlineStr"/>
       <c r="R43" t="inlineStr"/>
+      <c r="S43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -3108,6 +3155,7 @@
       <c r="P44" t="inlineStr"/>
       <c r="Q44" t="inlineStr"/>
       <c r="R44" t="inlineStr"/>
+      <c r="S44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -3166,6 +3214,7 @@
       <c r="P45" t="inlineStr"/>
       <c r="Q45" t="inlineStr"/>
       <c r="R45" t="inlineStr"/>
+      <c r="S45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -3224,6 +3273,7 @@
       <c r="P46" t="inlineStr"/>
       <c r="Q46" t="inlineStr"/>
       <c r="R46" t="inlineStr"/>
+      <c r="S46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -3282,6 +3332,7 @@
       <c r="P47" t="inlineStr"/>
       <c r="Q47" t="inlineStr"/>
       <c r="R47" t="inlineStr"/>
+      <c r="S47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -3340,6 +3391,7 @@
       <c r="P48" t="inlineStr"/>
       <c r="Q48" t="inlineStr"/>
       <c r="R48" t="inlineStr"/>
+      <c r="S48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -3398,6 +3450,7 @@
       <c r="P49" t="inlineStr"/>
       <c r="Q49" t="inlineStr"/>
       <c r="R49" t="inlineStr"/>
+      <c r="S49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -3456,6 +3509,7 @@
       <c r="P50" t="inlineStr"/>
       <c r="Q50" t="inlineStr"/>
       <c r="R50" t="inlineStr"/>
+      <c r="S50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -3514,6 +3568,7 @@
       <c r="P51" t="inlineStr"/>
       <c r="Q51" t="inlineStr"/>
       <c r="R51" t="inlineStr"/>
+      <c r="S51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -3572,6 +3627,7 @@
       <c r="P52" t="inlineStr"/>
       <c r="Q52" t="inlineStr"/>
       <c r="R52" t="inlineStr"/>
+      <c r="S52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -3630,6 +3686,7 @@
       <c r="P53" t="inlineStr"/>
       <c r="Q53" t="inlineStr"/>
       <c r="R53" t="inlineStr"/>
+      <c r="S53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -3688,6 +3745,7 @@
       <c r="P54" t="inlineStr"/>
       <c r="Q54" t="inlineStr"/>
       <c r="R54" t="inlineStr"/>
+      <c r="S54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -3746,6 +3804,7 @@
       <c r="P55" t="inlineStr"/>
       <c r="Q55" t="inlineStr"/>
       <c r="R55" t="inlineStr"/>
+      <c r="S55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -3804,6 +3863,7 @@
       <c r="P56" t="inlineStr"/>
       <c r="Q56" t="inlineStr"/>
       <c r="R56" t="inlineStr"/>
+      <c r="S56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -3862,6 +3922,7 @@
       <c r="P57" t="inlineStr"/>
       <c r="Q57" t="inlineStr"/>
       <c r="R57" t="inlineStr"/>
+      <c r="S57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -3920,6 +3981,7 @@
       <c r="P58" t="inlineStr"/>
       <c r="Q58" t="inlineStr"/>
       <c r="R58" t="inlineStr"/>
+      <c r="S58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -3978,6 +4040,7 @@
       <c r="P59" t="inlineStr"/>
       <c r="Q59" t="inlineStr"/>
       <c r="R59" t="inlineStr"/>
+      <c r="S59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -4036,6 +4099,7 @@
       <c r="P60" t="inlineStr"/>
       <c r="Q60" t="inlineStr"/>
       <c r="R60" t="inlineStr"/>
+      <c r="S60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -4094,6 +4158,7 @@
       <c r="P61" t="inlineStr"/>
       <c r="Q61" t="inlineStr"/>
       <c r="R61" t="inlineStr"/>
+      <c r="S61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -4152,6 +4217,7 @@
       <c r="P62" t="inlineStr"/>
       <c r="Q62" t="inlineStr"/>
       <c r="R62" t="inlineStr"/>
+      <c r="S62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -4210,6 +4276,7 @@
       <c r="P63" t="inlineStr"/>
       <c r="Q63" t="inlineStr"/>
       <c r="R63" t="inlineStr"/>
+      <c r="S63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -4268,6 +4335,7 @@
       <c r="P64" t="inlineStr"/>
       <c r="Q64" t="inlineStr"/>
       <c r="R64" t="inlineStr"/>
+      <c r="S64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -4326,6 +4394,7 @@
       <c r="P65" t="inlineStr"/>
       <c r="Q65" t="inlineStr"/>
       <c r="R65" t="inlineStr"/>
+      <c r="S65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -4384,6 +4453,7 @@
       <c r="P66" t="inlineStr"/>
       <c r="Q66" t="inlineStr"/>
       <c r="R66" t="inlineStr"/>
+      <c r="S66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -4442,6 +4512,7 @@
       <c r="P67" t="inlineStr"/>
       <c r="Q67" t="inlineStr"/>
       <c r="R67" t="inlineStr"/>
+      <c r="S67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -4500,6 +4571,7 @@
       <c r="P68" t="inlineStr"/>
       <c r="Q68" t="inlineStr"/>
       <c r="R68" t="inlineStr"/>
+      <c r="S68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -4558,6 +4630,7 @@
       <c r="P69" t="inlineStr"/>
       <c r="Q69" t="inlineStr"/>
       <c r="R69" t="inlineStr"/>
+      <c r="S69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -4616,6 +4689,7 @@
       <c r="P70" t="inlineStr"/>
       <c r="Q70" t="inlineStr"/>
       <c r="R70" t="inlineStr"/>
+      <c r="S70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -4674,6 +4748,7 @@
       <c r="P71" t="inlineStr"/>
       <c r="Q71" t="inlineStr"/>
       <c r="R71" t="inlineStr"/>
+      <c r="S71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -4732,6 +4807,7 @@
       <c r="P72" t="inlineStr"/>
       <c r="Q72" t="inlineStr"/>
       <c r="R72" t="inlineStr"/>
+      <c r="S72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -4790,6 +4866,7 @@
       <c r="P73" t="inlineStr"/>
       <c r="Q73" t="inlineStr"/>
       <c r="R73" t="inlineStr"/>
+      <c r="S73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -4848,6 +4925,7 @@
       <c r="P74" t="inlineStr"/>
       <c r="Q74" t="inlineStr"/>
       <c r="R74" t="inlineStr"/>
+      <c r="S74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -4906,6 +4984,7 @@
       <c r="P75" t="inlineStr"/>
       <c r="Q75" t="inlineStr"/>
       <c r="R75" t="inlineStr"/>
+      <c r="S75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -4964,6 +5043,7 @@
       <c r="P76" t="inlineStr"/>
       <c r="Q76" t="inlineStr"/>
       <c r="R76" t="inlineStr"/>
+      <c r="S76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -5022,6 +5102,7 @@
       <c r="P77" t="inlineStr"/>
       <c r="Q77" t="inlineStr"/>
       <c r="R77" t="inlineStr"/>
+      <c r="S77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -5080,6 +5161,7 @@
       <c r="P78" t="inlineStr"/>
       <c r="Q78" t="inlineStr"/>
       <c r="R78" t="inlineStr"/>
+      <c r="S78" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>